<commit_message>
reorder title of fig.
</commit_message>
<xml_diff>
--- a/outcome/publish/Table 3.xlsx
+++ b/outcome/publish/Table 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - kanggle\XMU\likangguo\other\github\zhuhai_omicron\outcome\publish\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21777B52-C100-4CFC-A41F-97FAFC672E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2945225-7276-4473-8018-FC3D57E8443F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
-  <si>
-    <t>mean</t>
-  </si>
-  <si>
-    <t>sd</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
   <si>
     <t>Generation time</t>
   </si>
@@ -52,10 +46,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Variant</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Omicron BA.1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -69,6 +59,22 @@
   </si>
   <si>
     <t>Rate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Variants</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Gamma distribution</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mean</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SD.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -76,6 +82,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -112,13 +121,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -400,264 +421,304 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.625" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="6" width="6.125" customWidth="1"/>
+    <col min="3" max="4" width="9.75" customWidth="1"/>
+    <col min="5" max="6" width="6.125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="5"/>
+      <c r="E1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
-        <v>1.64</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="E2" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="F2" s="1">
-        <v>4.45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2.12</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0.71</v>
-      </c>
-      <c r="E3" s="1">
-        <v>3</v>
-      </c>
-      <c r="F3" s="1">
-        <v>2.06</v>
-      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1.64</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="E4" s="6">
+        <v>5.7</v>
+      </c>
+      <c r="F4" s="6">
+        <v>4.45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="2"/>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="6">
+        <v>2.12</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="E5" s="6">
+        <v>3</v>
+      </c>
+      <c r="F5" s="6">
+        <v>2.06</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="6">
         <v>3.16</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D6" s="6">
         <v>1.41</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E6" s="6">
         <v>2.2400000000000002</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F6" s="6">
         <v>1.26</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="2"/>
+      <c r="B8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="6">
         <v>4.57</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D8" s="6">
         <v>0.6</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E8" s="6">
         <v>7.63</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F8" s="6">
         <v>3.57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="1">
-        <v>3.66</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.84</v>
-      </c>
-      <c r="E6" s="1">
-        <v>4.3499999999999996</v>
-      </c>
-      <c r="F6" s="1">
-        <v>2.27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1">
-        <v>3.42</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="E7" s="1">
-        <v>3.07</v>
-      </c>
-      <c r="F7" s="1">
-        <v>1.66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="1">
-        <v>1.18</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0.47</v>
-      </c>
-      <c r="E8" s="1">
-        <v>2.52</v>
-      </c>
-      <c r="F8" s="1">
-        <v>2.3199999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1">
-        <v>2.44</v>
-      </c>
-      <c r="D9" s="1">
-        <v>1.39</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1.76</v>
-      </c>
-      <c r="F9" s="1">
-        <v>1.1299999999999999</v>
+        <v>6</v>
+      </c>
+      <c r="C9" s="6">
+        <v>3.66</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0.84</v>
+      </c>
+      <c r="E9" s="6">
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="F9" s="6">
+        <v>2.27</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="2"/>
       <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1">
-        <v>6.59</v>
-      </c>
-      <c r="D10" s="1">
-        <v>2.25</v>
-      </c>
-      <c r="E10" s="1">
-        <v>2.93</v>
-      </c>
-      <c r="F10" s="1">
-        <v>1.1399999999999999</v>
+        <v>7</v>
+      </c>
+      <c r="C10" s="6">
+        <v>3.42</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="E10" s="6">
+        <v>3.07</v>
+      </c>
+      <c r="F10" s="6">
+        <v>1.66</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1.48</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0.41</v>
-      </c>
-      <c r="E11" s="1">
-        <v>3.61</v>
-      </c>
-      <c r="F11" s="1">
-        <v>2.97</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="1">
-        <v>3.17</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0.89</v>
-      </c>
-      <c r="E12" s="1">
-        <v>3.56</v>
-      </c>
-      <c r="F12" s="1">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C12" s="6">
+        <v>1.18</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0.47</v>
+      </c>
+      <c r="E12" s="6">
+        <v>2.52</v>
+      </c>
+      <c r="F12" s="6">
+        <v>2.3199999999999998</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="1">
+        <v>6</v>
+      </c>
+      <c r="C13" s="6">
+        <v>2.44</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1.39</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1.76</v>
+      </c>
+      <c r="F13" s="6">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="6">
+        <v>6.59</v>
+      </c>
+      <c r="D14" s="6">
+        <v>2.25</v>
+      </c>
+      <c r="E14" s="6">
+        <v>2.93</v>
+      </c>
+      <c r="F14" s="6">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1.48</v>
+      </c>
+      <c r="D16" s="6">
+        <v>0.41</v>
+      </c>
+      <c r="E16" s="6">
+        <v>3.61</v>
+      </c>
+      <c r="F16" s="6">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="2"/>
+      <c r="B17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="6">
+        <v>3.17</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.89</v>
+      </c>
+      <c r="E17" s="6">
+        <v>3.56</v>
+      </c>
+      <c r="F17" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="6">
         <v>3.6</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D18" s="6">
         <v>1.85</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E18" s="6">
         <v>1.95</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F18" s="6">
         <v>1.03</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A13"/>
+  <mergeCells count="5">
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>